<commit_message>
refactor: update evaluation labels and adjust budget example data
Standardize evaluation period labels in auswertung.go and update the
budget example configuration to reflect revised project financial
planning.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/output.xlsx
+++ b/sidecars/Vorpruefung/output.xlsx
@@ -6184,10 +6184,10 @@
         <v>500000</v>
       </c>
       <c r="G7" s="24">
-        <v>450000</v>
+        <v>437500</v>
       </c>
       <c r="H7" s="24">
-        <v>300000</v>
+        <v>312500</v>
       </c>
       <c r="I7" s="41">
         <v>10000</v>
@@ -6248,13 +6248,13 @@
         <f>=SUM(TblDrittmittel[Betrag (LC)])</f>
       </c>
       <c r="F10" s="24">
+        <v>1500000</v>
+      </c>
+      <c r="G10" s="24">
+        <v>1250000</v>
+      </c>
+      <c r="H10" s="24">
         <v>1000000</v>
-      </c>
-      <c r="G10" s="24">
-        <v>800000</v>
-      </c>
-      <c r="H10" s="24">
-        <v>700000</v>
       </c>
       <c r="I10" s="54" t="str">
         <f>=SUM(TblDrittmittel[Betrag (EUR)])</f>
@@ -6308,19 +6308,19 @@
         <v>199</v>
       </c>
       <c r="E13" s="24">
-        <v>6250000</v>
+        <v>7500000</v>
       </c>
       <c r="F13" s="24">
+        <v>3000000</v>
+      </c>
+      <c r="G13" s="24">
         <v>2500000</v>
       </c>
-      <c r="G13" s="24">
+      <c r="H13" s="24">
         <v>2000000</v>
       </c>
-      <c r="H13" s="24">
-        <v>1750000</v>
-      </c>
       <c r="I13" s="41">
-        <v>50000</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="14">
@@ -6416,28 +6416,28 @@
         <v>207</v>
       </c>
       <c r="E19" s="24">
-        <v>2000000</v>
+        <v>2500000</v>
       </c>
       <c r="F19" s="24">
-        <v>1200000</v>
+        <v>1500000</v>
       </c>
       <c r="G19" s="24">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="H19" s="24">
         <v>0</v>
       </c>
       <c r="I19" s="41">
-        <v>16000</v>
+        <v>20000</v>
       </c>
       <c r="K19" s="40" t="s">
         <v>235</v>
       </c>
       <c r="L19" s="24">
-        <v>1500000</v>
+        <v>2500000</v>
       </c>
       <c r="M19" s="41">
-        <v>12000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="20">
@@ -6451,28 +6451,28 @@
         <v>209</v>
       </c>
       <c r="E20" s="24">
-        <v>1000000</v>
+        <v>1250000</v>
       </c>
       <c r="F20" s="24">
         <v>0</v>
       </c>
       <c r="G20" s="24">
-        <v>600000</v>
+        <v>750000</v>
       </c>
       <c r="H20" s="24">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="I20" s="41">
-        <v>8000</v>
+        <v>10000</v>
       </c>
       <c r="K20" s="42" t="s">
         <v>236</v>
       </c>
       <c r="L20" s="43">
-        <v>1000000</v>
+        <v>1250000</v>
       </c>
       <c r="M20" s="44">
-        <v>8000</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="21">
@@ -6486,10 +6486,10 @@
         <v>212</v>
       </c>
       <c r="E21" s="24">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="F21" s="24">
-        <v>800000</v>
+        <v>1000000</v>
       </c>
       <c r="G21" s="24">
         <v>0</v>
@@ -6498,7 +6498,7 @@
         <v>0</v>
       </c>
       <c r="I21" s="41">
-        <v>6400</v>
+        <v>8000</v>
       </c>
     </row>
     <row r="22">
@@ -6512,19 +6512,19 @@
         <v>215</v>
       </c>
       <c r="E22" s="24">
-        <v>1500000</v>
+        <v>1875000</v>
       </c>
       <c r="F22" s="24">
-        <v>500000</v>
+        <v>625000</v>
       </c>
       <c r="G22" s="24">
-        <v>500000</v>
+        <v>625000</v>
       </c>
       <c r="H22" s="24">
-        <v>500000</v>
+        <v>625000</v>
       </c>
       <c r="I22" s="41">
-        <v>12000</v>
+        <v>15000</v>
       </c>
     </row>
     <row r="23">
@@ -6538,19 +6538,19 @@
         <v>217</v>
       </c>
       <c r="E23" s="24">
-        <v>1200000</v>
+        <v>1500000</v>
       </c>
       <c r="F23" s="24">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="G23" s="24">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="H23" s="24">
-        <v>400000</v>
+        <v>500000</v>
       </c>
       <c r="I23" s="41">
-        <v>9600</v>
+        <v>12000</v>
       </c>
     </row>
     <row r="24">
@@ -6564,19 +6564,19 @@
         <v>220</v>
       </c>
       <c r="E24" s="24">
-        <v>700000</v>
+        <v>1250000</v>
       </c>
       <c r="F24" s="24">
-        <v>300000</v>
+        <v>500000</v>
       </c>
       <c r="G24" s="24">
-        <v>250000</v>
+        <v>375000</v>
       </c>
       <c r="H24" s="24">
-        <v>150000</v>
+        <v>375000</v>
       </c>
       <c r="I24" s="41">
-        <v>5600</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="25">
@@ -6590,19 +6590,19 @@
         <v>223</v>
       </c>
       <c r="E25" s="24">
-        <v>400000</v>
+        <v>625000</v>
       </c>
       <c r="F25" s="24">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="G25" s="24">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="H25" s="24">
-        <v>100000</v>
+        <v>125000</v>
       </c>
       <c r="I25" s="41">
-        <v>3200</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="26">
@@ -6616,19 +6616,19 @@
         <v>226</v>
       </c>
       <c r="E26" s="24">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="F26" s="24">
         <v>0</v>
       </c>
       <c r="G26" s="24">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="H26" s="24">
         <v>0</v>
       </c>
       <c r="I26" s="41">
-        <v>1600</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="27">
@@ -6642,19 +6642,19 @@
         <v>229</v>
       </c>
       <c r="E27" s="24">
-        <v>150000</v>
+        <v>250000</v>
       </c>
       <c r="F27" s="24">
-        <v>50000</v>
+        <v>125000</v>
       </c>
       <c r="G27" s="24">
-        <v>50000</v>
+        <v>62500</v>
       </c>
       <c r="H27" s="24">
-        <v>50000</v>
+        <v>62500</v>
       </c>
       <c r="I27" s="41">
-        <v>1200</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="28">
@@ -6668,19 +6668,19 @@
         <v>230</v>
       </c>
       <c r="E28" s="24">
-        <v>300000</v>
+        <v>2000000</v>
       </c>
       <c r="F28" s="24">
-        <v>100000</v>
+        <v>625000</v>
       </c>
       <c r="G28" s="24">
-        <v>100000</v>
+        <v>625000</v>
       </c>
       <c r="H28" s="24">
-        <v>100000</v>
+        <v>750000</v>
       </c>
       <c r="I28" s="41">
-        <v>2400</v>
+        <v>16000</v>
       </c>
     </row>
     <row r="29" ht="20" customHeight="true">

</xml_diff>

<commit_message>
refactor: replace volatile INDIRECT with non-volatile CHOOSE
Replaced INDIRECT-based cell references with CHOOSE expressions to avoid
volatility and issues with Excel's implicit intersection operator.
</commit_message>
<xml_diff>
--- a/sidecars/Vorpruefung/output.xlsx
+++ b/sidecars/Vorpruefung/output.xlsx
@@ -150,7 +150,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="407">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="406" uniqueCount="406">
   <si>
     <t xml:space="preserve">  DASHBOARD (v1.0)</t>
   </si>
@@ -1187,7 +1187,7 @@
     <t>Neuste MA</t>
   </si>
   <si>
-    <t>Geprüfte Periode (FB+1)</t>
+    <t>Geprüfte Periode</t>
   </si>
   <si>
     <t>Ausgewählte Anforderung (#)</t>
@@ -1332,9 +1332,6 @@
   </si>
   <si>
     <t>Neuester FB</t>
-  </si>
-  <si>
-    <t>Geprüfte Periode (N)</t>
   </si>
   <si>
     <t>Saldo (LC)</t>
@@ -21738,7 +21735,7 @@
         <v>0</v>
       </c>
       <c r="L24" s="143" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="M24" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$21,'IV. MA'!$G$21,'IV. MA'!$K$21,'IV. MA'!$O$21,'IV. MA'!$S$21,'IV. MA'!$W$21,'IV. MA'!$AA$21,'IV. MA'!$AE$21,'IV. MA'!$AI$21,'IV. MA'!$AM$21,'IV. MA'!$AQ$21,'IV. MA'!$AU$21,'IV. MA'!$AY$21,'IV. MA'!$BC$21,'IV. MA'!$BG$21,'IV. MA'!$BK$21,'IV. MA'!$BO$21,'IV. MA'!$BS$21),"")</f>
@@ -21767,7 +21764,7 @@
         <v>0</v>
       </c>
       <c r="L25" s="143" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="M25" s="116" t="str">
         <f>=IFERROR(CHOOSE($AD$5,'IV. MA'!$C$22,'IV. MA'!$G$22,'IV. MA'!$K$22,'IV. MA'!$O$22,'IV. MA'!$S$22,'IV. MA'!$W$22,'IV. MA'!$AA$22,'IV. MA'!$AE$22,'IV. MA'!$AI$22,'IV. MA'!$AM$22,'IV. MA'!$AQ$22,'IV. MA'!$AU$22,'IV. MA'!$AY$22,'IV. MA'!$BC$22,'IV. MA'!$BG$22,'IV. MA'!$BK$22,'IV. MA'!$BO$22,'IV. MA'!$BS$22),"")</f>
@@ -21955,7 +21952,7 @@
         <f>=IFERROR(ROUND(CHOOSE(MATCH($D$41,{"Jahr 1";"Jahr 2";"Jahr 3"},0),SUBTOTAL(109,TblBudgetAusgaben[Jahr 1]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 2]),SUBTOTAL(109,TblBudgetAusgaben[Jahr 3])),2),0)</f>
       </c>
       <c r="E42" s="227" t="str">
-        <f>=IFERROR(ROUND($D$42/IFERROR(INDIRECT("MA_Kurs_"&amp;F10),0),2),0)</f>
+        <f>=IFERROR(ROUND($D$42/Budget_Kurs,2),0)</f>
       </c>
     </row>
     <row r="43">
@@ -22623,7 +22620,7 @@
     </row>
     <row r="82">
       <c r="C82" s="205" t="s">
-        <v>394</v>
+        <v>345</v>
       </c>
       <c r="D82" s="197"/>
       <c r="E82" s="197"/>
@@ -22645,12 +22642,12 @@
     </row>
     <row r="83">
       <c r="C83" s="205" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
       <c r="D83" s="197"/>
       <c r="E83" s="197"/>
       <c r="F83" s="241" t="str">
-        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoLC_"&amp;F82),2),0)</f>
+        <f>=IFERROR(ROUND(IFERROR(CHOOSE(F82,FB_SaldoLC_1,FB_SaldoLC_2,FB_SaldoLC_3,FB_SaldoLC_4,FB_SaldoLC_5,FB_SaldoLC_6,FB_SaldoLC_7,FB_SaldoLC_8,FB_SaldoLC_9,FB_SaldoLC_10,FB_SaldoLC_11,FB_SaldoLC_12,FB_SaldoLC_13,FB_SaldoLC_14,FB_SaldoLC_15,FB_SaldoLC_16,FB_SaldoLC_17,FB_SaldoLC_18),0),2),0)</f>
       </c>
       <c r="G83" s="241"/>
       <c r="H83" s="241"/>
@@ -22665,7 +22662,7 @@
       <c r="D84" s="255"/>
       <c r="E84" s="255"/>
       <c r="F84" s="289" t="str">
-        <f>=IFERROR(ROUND(INDIRECT("FB_SaldoEUR_"&amp;F82),2),0)</f>
+        <f>=IFERROR(ROUND(IFERROR(CHOOSE(F82,FB_SaldoEUR_1,FB_SaldoEUR_2,FB_SaldoEUR_3,FB_SaldoEUR_4,FB_SaldoEUR_5,FB_SaldoEUR_6,FB_SaldoEUR_7,FB_SaldoEUR_8,FB_SaldoEUR_9,FB_SaldoEUR_10,FB_SaldoEUR_11,FB_SaldoEUR_12,FB_SaldoEUR_13,FB_SaldoEUR_14,FB_SaldoEUR_15,FB_SaldoEUR_16,FB_SaldoEUR_17,FB_SaldoEUR_18),0),2),0)</f>
       </c>
       <c r="G84" s="289"/>
       <c r="H84" s="289"/>
@@ -22697,7 +22694,7 @@
     </row>
     <row r="86" ht="22" customHeight="true">
       <c r="B86" s="18" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="C86" s="18"/>
       <c r="D86" s="18"/>
@@ -22948,7 +22945,7 @@
     </row>
     <row r="96" ht="22" customHeight="true">
       <c r="B96" s="18" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C96" s="18"/>
       <c r="D96" s="18"/>
@@ -22996,7 +22993,7 @@
         <v>380</v>
       </c>
       <c r="C98" s="265" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D98" s="265" t="s">
         <v>382</v>
@@ -23008,7 +23005,7 @@
         <v>384</v>
       </c>
       <c r="G98" s="265" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="H98" s="265" t="s">
         <v>386</v>
@@ -23274,7 +23271,7 @@
     </row>
     <row r="105" ht="22" customHeight="true">
       <c r="B105" s="18" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
       <c r="C105" s="18"/>
       <c r="D105" s="18"/>
@@ -23309,7 +23306,7 @@
         <v>380</v>
       </c>
       <c r="C107" s="265" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="D107" s="265" t="s">
         <v>382</v>
@@ -23321,7 +23318,7 @@
         <v>384</v>
       </c>
       <c r="G107" s="265" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
       <c r="H107" s="265" t="s">
         <v>386</v>
@@ -23906,16 +23903,16 @@
         <v>247</v>
       </c>
       <c r="C1" s="352" t="s">
+        <v>402</v>
+      </c>
+      <c r="I1" s="352" t="s">
         <v>403</v>
       </c>
-      <c r="I1" s="352" t="s">
+      <c r="O1" s="352" t="s">
         <v>404</v>
       </c>
-      <c r="O1" s="352" t="s">
+      <c r="U1" s="352" t="s">
         <v>405</v>
-      </c>
-      <c r="U1" s="352" t="s">
-        <v>406</v>
       </c>
       <c r="BA1">
         <v>1</v>

</xml_diff>